<commit_message>
added the excel data validation
</commit_message>
<xml_diff>
--- a/excel/interest-data.xlsx
+++ b/excel/interest-data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I29"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -874,9 +874,63 @@
         <v>13167</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Car Loan</v>
+      </c>
+      <c r="B27" t="str">
+        <v>800000</v>
+      </c>
+      <c r="C27" t="str">
+        <v>9</v>
+      </c>
+      <c r="D27" t="str">
+        <v>5</v>
+      </c>
+      <c r="H27" t="str">
+        <v>69961</v>
+      </c>
+      <c r="I27" t="str">
+        <v>16483</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Home Loan</v>
+      </c>
+      <c r="B28" t="str">
+        <v>1000000</v>
+      </c>
+      <c r="C28" t="str">
+        <v>8.5</v>
+      </c>
+      <c r="D28" t="str">
+        <v>20</v>
+      </c>
+      <c r="E28">
+        <v>8678</v>
+      </c>
+      <c r="F28" t="str">
+        <v>10,82,776</v>
+      </c>
+      <c r="G28" t="str">
+        <v>20,82,776</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Personal Loan</v>
+      </c>
+      <c r="B29" t="str">
+        <v>500000</v>
+      </c>
+      <c r="E29">
+        <v>13167</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I29"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>